<commit_message>
fix: solar pv `active_area_fraction`
</commit_message>
<xml_diff>
--- a/src/cubes/data/energy_systems/solar-pv.xlsx
+++ b/src/cubes/data/energy_systems/solar-pv.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10409"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10514"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottjeen/phd/research/CUBES/src/cubes/data/energy_systems/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF467A94-2C2B-E945-B366-79EB2AA93F74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7FDAF6E-EE1E-BD49-8D54-42DACEA057A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3080" yWindow="4040" windowWidth="28040" windowHeight="17440" xr2:uid="{6613BF47-8E0B-1F4E-9D7F-2739A296C47F}"/>
   </bookViews>
@@ -143,13 +143,13 @@
     <t>COUNTRY SOLAR PV INSTALLATIONS</t>
   </si>
   <si>
-    <t>MEAN SOLAR PV ACTIVE AREA FRACTION</t>
-  </si>
-  <si>
     <t>SOLAR PV TECHNICAL POTENTIAL INSTALLATIONS</t>
   </si>
   <si>
     <t>MEAN SOLAR PV PANEL EFFICIENCY</t>
+  </si>
+  <si>
+    <t>SOLAR PV ACTIVE AREA FRACTION</t>
   </si>
 </sst>
 </file>
@@ -556,13 +556,13 @@
         <v>34</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -576,7 +576,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E7" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -590,7 +590,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E8" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -604,7 +604,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E9" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -618,7 +618,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E10" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -632,7 +632,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E11" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -646,7 +646,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E12" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -660,7 +660,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E13" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -674,7 +674,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E14" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -688,7 +688,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E15" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
@@ -702,7 +702,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E16" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -716,7 +716,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E17" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -730,7 +730,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E18" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -744,7 +744,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E19" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -758,7 +758,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E20" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -772,7 +772,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E21" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -786,7 +786,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E22" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
@@ -800,7 +800,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E23" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
@@ -814,7 +814,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E24" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
@@ -828,7 +828,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E25" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
@@ -842,7 +842,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E26" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -856,7 +856,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E27" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -870,7 +870,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E28" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -884,7 +884,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E29" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -898,7 +898,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E30" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -912,7 +912,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E31" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -926,7 +926,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E32" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -940,7 +940,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E33" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
@@ -957,7 +957,7 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="E34" s="3">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>